<commit_message>
change in table and graphs by model update 1.1
</commit_message>
<xml_diff>
--- a/output/coefficients/comparison_table.xlsx
+++ b/output/coefficients/comparison_table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,27 +456,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.1115 (11.8%)</t>
+          <t>0.1076 (11.36%)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.0784 (8.16%)</t>
+          <t>0.0756 (7.85%)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.0127 (1.28%)</t>
+          <t>0.0116 (1.17%)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.0579 (5.96%)</t>
+          <t>0.0561 (5.77%)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.0259 (2.62%)</t>
+          <t>0.025 (2.53%)</t>
         </is>
       </c>
     </row>
@@ -488,703 +488,799 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>-0.2647 (-23.25%)</t>
+          <t>-0.2455 (-21.77%)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>-0.1549 (-14.35%)</t>
+          <t>-0.1424 (-13.27%)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>-0.0178 (-1.76%)</t>
+          <t>-0.0134 (-1.33%)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-0.1165 (-11.0%)</t>
+          <t>-0.1091 (-10.34%)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>-0.0537 (-5.23%)</t>
+          <t>-0.0502 (-4.89%)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>d_action</t>
+          <t>d_aa</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.0663 (6.86%)</t>
+          <t>-0.0889 (-8.5%)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.0633 (6.53%)</t>
+          <t>-0.0598 (-5.8%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-0.0207 (-2.05%)</t>
+          <t>-0.0306 (-3.01%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.0625 (6.45%)</t>
+          <t>-0.046 (-4.5%)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.0266 (2.7%)</t>
+          <t>-0.0183 (-1.81%)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>d_actionadventure</t>
+          <t>d_action</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.115 (12.18%)</t>
+          <t>0.0529 (5.43%)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.066 (6.82%)</t>
+          <t>0.0548 (5.63%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-0.0315 (-3.1%)</t>
+          <t>-0.0276 (-2.73%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.0879 (9.19%)</t>
+          <t>0.0562 (5.78%)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.0298 (3.02%)</t>
+          <t>0.0243 (2.46%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d_adventure</t>
+          <t>d_actionadventure</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>-0.0034 (-0.34%)</t>
+          <t>0.0912 (9.55%)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.0343 (3.49%)</t>
+          <t>0.051 (5.23%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-0.0566 (-5.5%)</t>
+          <t>-0.042 (-4.12%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.0447 (4.57%)</t>
+          <t>0.0773 (8.03%)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.0202 (2.04%)</t>
+          <t>0.0253 (2.56%)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>d_fighting</t>
+          <t>d_adventure</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.0402 (4.11%)</t>
+          <t>0.0099 (0.99%)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.0561 (5.77%)</t>
+          <t>0.0348 (3.54%)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-0.0282 (-2.78%)</t>
+          <t>-0.0495 (-4.83%)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.0324 (3.3%)</t>
+          <t>0.0453 (4.63%)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.0171 (1.73%)</t>
+          <t>0.021 (2.12%)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>d_misc</t>
+          <t>d_fighting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0.0625 (6.45%)</t>
+          <t>0.0347 (3.53%)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.0772 (8.03%)</t>
+          <t>0.0555 (5.7%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-0.0278 (-2.74%)</t>
+          <t>-0.0294 (-2.9%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.0674 (6.97%)</t>
+          <t>0.0321 (3.26%)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0.0325 (3.31%)</t>
+          <t>0.0174 (1.76%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>d_mshome</t>
+          <t>d_indie</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>-0.0432 (-4.23%)</t>
+          <t>-0.065 (-6.29%)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.0089 (0.89%)</t>
+          <t>-0.0427 (-4.18%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.0713 (-6.88%)</t>
+          <t>-0.0367 (-3.61%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>-0.0703 (-6.79%)</t>
+          <t>-0.0306 (-3.02%)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>-0.048 (-4.69%)</t>
+          <t>-0.0173 (-1.72%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>d_music</t>
+          <t>d_misc</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0.0863 (9.01%)</t>
+          <t>0.0592 (6.09%)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.0742 (7.7%)</t>
+          <t>0.0732 (7.6%)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.0244 (2.47%)</t>
+          <t>-0.0277 (-2.73%)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.0542 (5.57%)</t>
+          <t>0.0641 (6.62%)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.0165 (1.66%)</t>
+          <t>0.0313 (3.18%)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>d_nintendohandheld</t>
+          <t>d_mshome</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>-0.1311 (-12.29%)</t>
+          <t>-0.0467 (-4.56%)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>-0.0612 (-5.94%)</t>
+          <t>0.0062 (0.63%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.0023 (0.23%)</t>
+          <t>-0.0719 (-6.93%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>-0.1022 (-9.71%)</t>
+          <t>-0.0711 (-6.87%)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>-0.0599 (-5.82%)</t>
+          <t>-0.0485 (-4.74%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>d_nintendohome</t>
+          <t>d_music</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>-0.1108 (-10.48%)</t>
+          <t>0.0602 (6.2%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-0.0435 (-4.26%)</t>
+          <t>0.0553 (5.69%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.0242 (-2.39%)</t>
+          <t>0.0181 (1.82%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-0.1019 (-9.69%)</t>
+          <t>0.0414 (4.23%)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.0587 (-5.7%)</t>
+          <t>0.011 (1.1%)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>d_other</t>
+          <t>d_nintendohandheld</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0.0565 (5.82%)</t>
+          <t>-0.1202 (-11.32%)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.0323 (3.28%)</t>
+          <t>-0.0504 (-4.91%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.029 (2.94%)</t>
+          <t>0.0023 (0.23%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.0468 (4.79%)</t>
+          <t>-0.0955 (-9.11%)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.0091 (0.91%)</t>
+          <t>-0.0568 (-5.52%)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>d_pcmac</t>
+          <t>d_nintendohome</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>-0.2373 (-21.12%)</t>
+          <t>-0.1018 (-9.68%)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-0.1573 (-14.55%)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>-0.0358 (-3.52%)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>-0.0266 (-2.63%)</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>-0.1215 (-11.44%)</t>
+          <t>-0.0973 (-9.27%)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>-0.0725 (-6.99%)</t>
+          <t>-0.0563 (-5.47%)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>d_platform</t>
+          <t>d_other</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0.0556 (5.72%)</t>
+          <t>0.0165 (1.66%)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>0.0385 (3.93%)</t>
+          <t>0.009 (0.9%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-0.0336 (-3.31%)</t>
+          <t>0.0158 (1.59%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.0564 (5.8%)</t>
+          <t>0.0309 (3.13%)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.0206 (2.08%)</t>
+          <t>0.0015 (0.15%)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>d_puzzle</t>
+          <t>d_pcmac</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>-0.0015 (-0.15%)</t>
+          <t>-0.2341 (-20.87%)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.005 (0.5%)</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>-0.034 (-3.34%)</t>
-        </is>
-      </c>
+          <t>-0.1594 (-14.73%)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.0273 (2.77%)</t>
+          <t>-0.1178 (-11.11%)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.0149 (1.5%)</t>
+          <t>-0.0714 (-6.89%)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>d_racing</t>
+          <t>d_platform</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0.044 (4.5%)</t>
+          <t>0.0434 (4.44%)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.0244 (2.47%)</t>
+          <t>0.0309 (3.14%)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>-0.0679 (-6.57%)</t>
+          <t>-0.0439 (-4.3%)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.0624 (6.44%)</t>
+          <t>0.0504 (5.17%)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.0212 (2.14%)</t>
+          <t>0.0186 (1.87%)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>d_sega</t>
+          <t>d_puzzle</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>-0.3082 (-26.52%)</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
+          <t>0.0118 (1.19%)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>0.0171 (1.72%)</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>-0.0041 (-0.4%)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
+          <t>-0.0412 (-4.03%)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.0323 (3.28%)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.0178 (1.8%)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>d_shooter</t>
+          <t>d_racing</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0.14 (15.03%)</t>
+          <t>0.0449 (4.59%)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.1112 (11.76%)</t>
+          <t>0.0255 (2.59%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>-0.0371 (-3.65%)</t>
+          <t>-0.0709 (-6.84%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.1096 (11.59%)</t>
+          <t>0.0616 (6.36%)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0.0467 (4.78%)</t>
+          <t>0.022 (2.22%)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>d_simulation</t>
+          <t>d_sega</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0.0736 (7.63%)</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>0.0776 (8.07%)</t>
-        </is>
-      </c>
+          <t>-0.3222 (-27.54%)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>-0.0342 (-3.37%)</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>0.0754 (7.83%)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>0.0276 (2.8%)</t>
-        </is>
-      </c>
+          <t>-0.0086 (-0.86%)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>d_sonyhandheld</t>
+          <t>d_shooter</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>-0.1596 (-14.75%)</t>
+          <t>0.1313 (14.03%)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>-0.1039 (-9.87%)</t>
+          <t>0.1057 (11.15%)</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>-0.0178 (-1.77%)</t>
+          <t>-0.0439 (-4.3%)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>-0.1014 (-9.64%)</t>
+          <t>0.1042 (10.98%)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>-0.0357 (-3.51%)</t>
+          <t>0.0449 (4.59%)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>d_sports</t>
+          <t>d_simulation</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0.0966 (10.15%)</t>
+          <t>0.0642 (6.63%)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.0807 (8.4%)</t>
+          <t>0.0697 (7.22%)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>-0.0014 (-0.14%)</t>
+          <t>-0.0344 (-3.38%)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0.0711 (7.37%)</t>
+          <t>0.0681 (7.05%)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0.0333 (3.39%)</t>
+          <t>0.0254 (2.57%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>d_strategy</t>
+          <t>d_sonyhandheld</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>-0.0302 (-2.97%)</t>
+          <t>-0.1491 (-13.85%)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>-0.0274 (-2.71%)</t>
+          <t>-0.1041 (-9.88%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>-0.0093 (-0.93%)</t>
+          <t>-0.013 (-1.29%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.0106 (1.07%)</t>
+          <t>-0.1016 (-9.66%)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.0049 (0.49%)</t>
+          <t>-0.0355 (-3.49%)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>d_visualnovel</t>
+          <t>d_sports</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>-0.0626 (-6.07%)</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>0.0706 (7.32%)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0.0634 (6.54%)</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>-0.049 (-4.78%)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
+          <t>-0.0145 (-1.44%)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>0.0594 (6.12%)</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0.0286 (2.9%)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>d_strategy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>-0.0391 (-3.83%)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>-0.0307 (-3.02%)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>-0.0156 (-1.54%)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0.0067 (0.67%)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0.0037 (0.37%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>d_unknown</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>-0.1334 (-12.49%)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>-0.0973 (-9.27%)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>-0.0375 (-3.68%)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>-0.0586 (-5.69%)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>-0.0245 (-2.42%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>d_visualnovel</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>-0.0266 (-2.63%)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>-0.0375 (-3.68%)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>year_c</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>-0.0012 (-0.12%)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>-0.0013 (-0.13%)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>-0.0044 (-0.44%)</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>0.0055 (0.56%)</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>0.0018 (0.18%)</t>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>-0.0015 (-0.15%)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>-0.0017 (-0.17%)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>-0.0043 (-0.43%)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>0.005 (0.5%)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>0.0017 (0.17%)</t>
         </is>
       </c>
     </row>

</xml_diff>